<commit_message>
Fix LEAN regex, add auto_compare.py, nightly file-check task
</commit_message>
<xml_diff>
--- a/flask_backend/test_output/result_table_v2.xlsx
+++ b/flask_backend/test_output/result_table_v2.xlsx
@@ -3078,7 +3078,7 @@
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -3373,7 +3373,7 @@
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -3403,7 +3403,7 @@
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -7389,7 +7389,7 @@
     <row r="240" ht="14" customHeight="1">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B240" s="5" t="inlineStr">
@@ -7719,7 +7719,7 @@
     <row r="251" ht="14" customHeight="1">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B251" s="5" t="inlineStr">
@@ -7779,7 +7779,7 @@
     <row r="253" ht="14" customHeight="1">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B253" s="5" t="inlineStr">
@@ -7809,7 +7809,7 @@
     <row r="254" ht="14" customHeight="1">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B254" s="5" t="inlineStr">
@@ -7895,7 +7895,7 @@
     <row r="257" ht="14" customHeight="1">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B257" s="5" t="inlineStr">
@@ -7925,7 +7925,7 @@
     <row r="258" ht="14" customHeight="1">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B258" s="5" t="inlineStr">
@@ -8516,7 +8516,7 @@
     <row r="279" ht="14" customHeight="1">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B279" s="5" t="inlineStr">
@@ -8876,7 +8876,7 @@
     <row r="291" ht="14" customHeight="1">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B291" s="5" t="inlineStr">
@@ -11795,7 +11795,7 @@
     <row r="395" ht="14" customHeight="1">
       <c r="A395" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B395" s="5" t="inlineStr">
@@ -11825,7 +11825,7 @@
     <row r="396" ht="14" customHeight="1">
       <c r="A396" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B396" s="5" t="inlineStr">
@@ -11855,7 +11855,7 @@
     <row r="397" ht="14" customHeight="1">
       <c r="A397" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B397" s="5" t="inlineStr">
@@ -11885,7 +11885,7 @@
     <row r="398" ht="14" customHeight="1">
       <c r="A398" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B398" s="5" t="inlineStr">
@@ -11915,7 +11915,7 @@
     <row r="399" ht="14" customHeight="1">
       <c r="A399" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B399" s="5" t="inlineStr">
@@ -11945,7 +11945,7 @@
     <row r="400" ht="14" customHeight="1">
       <c r="A400" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B400" s="5" t="inlineStr">
@@ -11975,7 +11975,7 @@
     <row r="401" ht="14" customHeight="1">
       <c r="A401" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B401" s="5" t="inlineStr">
@@ -12005,7 +12005,7 @@
     <row r="402" ht="14" customHeight="1">
       <c r="A402" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B402" s="5" t="inlineStr">
@@ -12035,7 +12035,7 @@
     <row r="403" ht="14" customHeight="1">
       <c r="A403" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B403" s="5" t="inlineStr">
@@ -12065,7 +12065,7 @@
     <row r="404" ht="14" customHeight="1">
       <c r="A404" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B404" s="5" t="inlineStr">
@@ -12147,7 +12147,7 @@
     <row r="407" ht="14" customHeight="1">
       <c r="A407" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B407" s="5" t="inlineStr">
@@ -12177,7 +12177,7 @@
     <row r="408" ht="14" customHeight="1">
       <c r="A408" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B408" s="5" t="inlineStr">
@@ -12207,7 +12207,7 @@
     <row r="409" ht="14" customHeight="1">
       <c r="A409" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B409" s="5" t="inlineStr">
@@ -12237,7 +12237,7 @@
     <row r="410" ht="14" customHeight="1">
       <c r="A410" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B410" s="5" t="inlineStr">
@@ -12267,7 +12267,7 @@
     <row r="411" ht="14" customHeight="1">
       <c r="A411" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B411" s="5" t="inlineStr">
@@ -12297,7 +12297,7 @@
     <row r="412" ht="14" customHeight="1">
       <c r="A412" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B412" s="5" t="inlineStr">
@@ -12327,7 +12327,7 @@
     <row r="413" ht="14" customHeight="1">
       <c r="A413" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B413" s="5" t="inlineStr">
@@ -12357,7 +12357,7 @@
     <row r="414" ht="14" customHeight="1">
       <c r="A414" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B414" s="5" t="inlineStr">
@@ -12387,7 +12387,7 @@
     <row r="415" ht="14" customHeight="1">
       <c r="A415" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B415" s="5" t="inlineStr">
@@ -12417,7 +12417,7 @@
     <row r="416" ht="14" customHeight="1">
       <c r="A416" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B416" s="5" t="inlineStr">
@@ -12447,7 +12447,7 @@
     <row r="417" ht="14" customHeight="1">
       <c r="A417" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B417" s="5" t="inlineStr">
@@ -12477,7 +12477,7 @@
     <row r="418" ht="14" customHeight="1">
       <c r="A418" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B418" s="5" t="inlineStr">
@@ -12507,7 +12507,7 @@
     <row r="419" ht="14" customHeight="1">
       <c r="A419" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B419" s="5" t="inlineStr">
@@ -12537,7 +12537,7 @@
     <row r="420" ht="14" customHeight="1">
       <c r="A420" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B420" s="5" t="inlineStr">
@@ -12567,7 +12567,7 @@
     <row r="421" ht="14" customHeight="1">
       <c r="A421" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B421" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
     <row r="422" ht="14" customHeight="1">
       <c r="A422" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B422" s="5" t="inlineStr">
@@ -12627,7 +12627,7 @@
     <row r="423" ht="14" customHeight="1">
       <c r="A423" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B423" s="5" t="inlineStr">
@@ -12657,7 +12657,7 @@
     <row r="424" ht="14" customHeight="1">
       <c r="A424" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B424" s="5" t="inlineStr">
@@ -12687,7 +12687,7 @@
     <row r="425" ht="14" customHeight="1">
       <c r="A425" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B425" s="5" t="inlineStr">
@@ -12717,7 +12717,7 @@
     <row r="426" ht="14" customHeight="1">
       <c r="A426" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B426" s="5" t="inlineStr">
@@ -12747,7 +12747,7 @@
     <row r="427" ht="14" customHeight="1">
       <c r="A427" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B427" s="5" t="inlineStr">
@@ -12807,7 +12807,7 @@
     <row r="429" ht="14" customHeight="1">
       <c r="A429" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B429" s="5" t="inlineStr">
@@ -12837,7 +12837,7 @@
     <row r="430" ht="14" customHeight="1">
       <c r="A430" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B430" s="5" t="inlineStr">
@@ -12893,7 +12893,7 @@
     <row r="432" ht="14" customHeight="1">
       <c r="A432" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B432" s="5" t="inlineStr">
@@ -12923,7 +12923,7 @@
     <row r="433" ht="14" customHeight="1">
       <c r="A433" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B433" s="5" t="inlineStr">
@@ -13005,7 +13005,7 @@
     <row r="436" ht="14" customHeight="1">
       <c r="A436" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B436" s="5" t="inlineStr">
@@ -13035,7 +13035,7 @@
     <row r="437" ht="14" customHeight="1">
       <c r="A437" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B437" s="5" t="inlineStr">
@@ -13065,7 +13065,7 @@
     <row r="438" ht="14" customHeight="1">
       <c r="A438" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B438" s="5" t="inlineStr">
@@ -13184,7 +13184,7 @@
     <row r="443" ht="14" customHeight="1">
       <c r="A443" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B443" s="5" t="inlineStr">
@@ -13214,7 +13214,7 @@
     <row r="444" ht="14" customHeight="1">
       <c r="A444" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B444" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
     <row r="445" ht="14" customHeight="1">
       <c r="A445" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B445" s="5" t="inlineStr">
@@ -13304,7 +13304,7 @@
     <row r="447" ht="14" customHeight="1">
       <c r="A447" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B447" s="5" t="inlineStr">
@@ -13334,7 +13334,7 @@
     <row r="448" ht="14" customHeight="1">
       <c r="A448" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B448" s="5" t="inlineStr">
@@ -13364,7 +13364,7 @@
     <row r="449" ht="14" customHeight="1">
       <c r="A449" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B449" s="5" t="inlineStr">
@@ -13394,7 +13394,7 @@
     <row r="450" ht="14" customHeight="1">
       <c r="A450" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B450" s="5" t="inlineStr">
@@ -21850,7 +21850,7 @@
     <row r="179" ht="14" customHeight="1">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
@@ -21878,7 +21878,7 @@
     <row r="180" ht="14" customHeight="1">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B180" s="5" t="inlineStr">
@@ -21906,7 +21906,7 @@
     <row r="181" ht="14" customHeight="1">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
@@ -21934,7 +21934,7 @@
     <row r="182" ht="14" customHeight="1">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B182" s="5" t="inlineStr">
@@ -21964,7 +21964,7 @@
     <row r="183" ht="14" customHeight="1">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
@@ -21994,7 +21994,7 @@
     <row r="184" ht="14" customHeight="1">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B184" s="5" t="inlineStr">
@@ -22024,7 +22024,7 @@
     <row r="185" ht="14" customHeight="1">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B185" s="5" t="inlineStr">
@@ -22054,7 +22054,7 @@
     <row r="186" ht="14" customHeight="1">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B186" s="5" t="inlineStr">
@@ -22084,7 +22084,7 @@
     <row r="187" ht="14" customHeight="1">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B187" s="5" t="inlineStr">
@@ -22114,7 +22114,7 @@
     <row r="188" ht="14" customHeight="1">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B188" s="5" t="inlineStr">
@@ -22144,7 +22144,7 @@
     <row r="189" ht="14" customHeight="1">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B189" s="5" t="inlineStr">
@@ -22172,7 +22172,7 @@
     <row r="190" ht="14" customHeight="1">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B190" s="5" t="inlineStr">
@@ -22202,7 +22202,7 @@
     <row r="191" ht="14" customHeight="1">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B191" s="5" t="inlineStr">
@@ -22230,7 +22230,7 @@
     <row r="192" ht="14" customHeight="1">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B192" s="5" t="inlineStr">
@@ -22258,7 +22258,7 @@
     <row r="193" ht="14" customHeight="1">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr">
@@ -22286,7 +22286,7 @@
     <row r="194" ht="14" customHeight="1">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B194" s="5" t="inlineStr">
@@ -22314,7 +22314,7 @@
     <row r="195" ht="14" customHeight="1">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr">
@@ -22344,7 +22344,7 @@
     <row r="196" ht="14" customHeight="1">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B196" s="5" t="inlineStr">
@@ -22374,7 +22374,7 @@
     <row r="197" ht="14" customHeight="1">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B197" s="5" t="inlineStr">
@@ -22404,7 +22404,7 @@
     <row r="198" ht="14" customHeight="1">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B198" s="5" t="inlineStr">
@@ -22434,7 +22434,7 @@
     <row r="199" ht="14" customHeight="1">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B199" s="5" t="inlineStr">
@@ -22464,7 +22464,7 @@
     <row r="200" ht="14" customHeight="1">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B200" s="5" t="inlineStr">
@@ -22494,7 +22494,7 @@
     <row r="201" ht="14" customHeight="1">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B201" s="5" t="inlineStr">
@@ -22524,7 +22524,7 @@
     <row r="202" ht="14" customHeight="1">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B202" s="5" t="inlineStr">
@@ -22552,7 +22552,7 @@
     <row r="203" ht="14" customHeight="1">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B203" s="5" t="inlineStr">
@@ -22580,7 +22580,7 @@
     <row r="204" ht="14" customHeight="1">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B204" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Fix LEAN source: read from DS-04 group titles instead of bianche
- Add _parse_lean_title() to convert 加一A组->1A, 加十一A1组->11A1
- load_schedule() now tracks art_lean per sheet from DS-04 col1 headers
- build_csa() uses per-sheet art_lean (no longer reads bianche for LEAN)
- build_v2.py: auto-copy locked source files to temp before loading
- Result: 301 LEAN consistent vs 272 before (+29 corrected)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flask_backend/test_output/result_table_v2.xlsx
+++ b/flask_backend/test_output/result_table_v2.xlsx
@@ -651,7 +651,7 @@
     <row r="4" ht="14" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2C</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2C</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2C</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1011,7 +1011,7 @@
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1071,7 +1071,7 @@
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1131,7 +1131,7 @@
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1159,7 +1159,11 @@
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="11" t="inlineStr"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
           <t>CODECHAOS 27</t>
@@ -1217,7 +1221,7 @@
     <row r="23" ht="14" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1307,7 +1311,7 @@
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1337,7 +1341,7 @@
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1367,7 +1371,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1397,7 +1401,7 @@
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1697,7 +1701,7 @@
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1845,7 +1849,11 @@
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="11" t="inlineStr"/>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -1871,7 +1879,11 @@
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="A45" s="11" t="inlineStr"/>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -1897,7 +1909,11 @@
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="11" t="inlineStr"/>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -2560,7 +2576,11 @@
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
-      <c r="A69" s="11" t="inlineStr"/>
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
           <t>MEGARIDE F50</t>
@@ -2826,7 +2846,11 @@
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="A78" s="11" t="inlineStr"/>
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
           <t>MEGARIDE F50</t>
@@ -2882,7 +2906,11 @@
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="A80" s="11" t="inlineStr"/>
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BOOT W</t>
@@ -2908,7 +2936,11 @@
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
-      <c r="A81" s="11" t="inlineStr"/>
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BOOT W</t>
@@ -3024,7 +3056,11 @@
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
-      <c r="A85" s="11" t="inlineStr"/>
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>2C</t>
+        </is>
+      </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -3050,7 +3086,11 @@
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
-      <c r="A86" s="11" t="inlineStr"/>
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>2C</t>
+        </is>
+      </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -3078,7 +3118,7 @@
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -3226,7 +3266,11 @@
       </c>
     </row>
     <row r="92" ht="14" customHeight="1">
-      <c r="A92" s="11" t="inlineStr"/>
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -3252,7 +3296,11 @@
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
-      <c r="A93" s="11" t="inlineStr"/>
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -3278,7 +3326,11 @@
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
-      <c r="A94" s="11" t="inlineStr"/>
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -3343,7 +3395,7 @@
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3373,7 +3425,7 @@
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>11B2</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -3403,7 +3455,7 @@
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>11B2</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3431,7 +3483,11 @@
       </c>
     </row>
     <row r="100" ht="14" customHeight="1">
-      <c r="A100" s="11" t="inlineStr"/>
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
           <t>OZWEEGO J</t>
@@ -3459,7 +3515,7 @@
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3489,7 +3545,7 @@
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>8A</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -3549,7 +3605,7 @@
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>3A</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -3579,7 +3635,7 @@
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>3A</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3609,7 +3665,7 @@
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>3A</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -3759,7 +3815,7 @@
     <row r="111" ht="14" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>3A</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -3819,7 +3875,7 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -3847,7 +3903,11 @@
       </c>
     </row>
     <row r="114" ht="14" customHeight="1">
-      <c r="A114" s="11" t="inlineStr"/>
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -3875,7 +3935,7 @@
     <row r="115" ht="14" customHeight="1">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -3995,7 +4055,7 @@
     <row r="119" ht="14" customHeight="1">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -4025,7 +4085,7 @@
     <row r="120" ht="14" customHeight="1">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
@@ -4053,7 +4113,11 @@
       </c>
     </row>
     <row r="121" ht="14" customHeight="1">
-      <c r="A121" s="11" t="inlineStr"/>
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -4139,7 +4203,11 @@
       </c>
     </row>
     <row r="124" ht="14" customHeight="1">
-      <c r="A124" s="11" t="inlineStr"/>
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -4165,7 +4233,11 @@
       </c>
     </row>
     <row r="125" ht="14" customHeight="1">
-      <c r="A125" s="11" t="inlineStr"/>
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -4191,7 +4263,11 @@
       </c>
     </row>
     <row r="126" ht="14" customHeight="1">
-      <c r="A126" s="11" t="inlineStr"/>
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -4217,7 +4293,11 @@
       </c>
     </row>
     <row r="127" ht="14" customHeight="1">
-      <c r="A127" s="11" t="inlineStr"/>
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -4243,7 +4323,11 @@
       </c>
     </row>
     <row r="128" ht="14" customHeight="1">
-      <c r="A128" s="11" t="inlineStr"/>
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -4278,7 +4362,7 @@
     <row r="130" ht="14" customHeight="1">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B130" s="5" t="inlineStr">
@@ -4338,7 +4422,7 @@
     <row r="132" ht="14" customHeight="1">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>5B</t>
         </is>
       </c>
       <c r="B132" s="5" t="inlineStr">
@@ -4366,7 +4450,11 @@
       </c>
     </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="A133" s="11" t="inlineStr"/>
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>5C</t>
+        </is>
+      </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
           <t>SL 72 RTN</t>
@@ -4452,7 +4540,11 @@
       </c>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="A136" s="11" t="inlineStr"/>
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>5C</t>
+        </is>
+      </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
@@ -4628,7 +4720,11 @@
       </c>
     </row>
     <row r="142" ht="14" customHeight="1">
-      <c r="A142" s="11" t="inlineStr"/>
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>5C</t>
+        </is>
+      </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
@@ -4656,7 +4752,7 @@
     <row r="143" ht="14" customHeight="1">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
@@ -4686,7 +4782,7 @@
     <row r="144" ht="14" customHeight="1">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B144" s="5" t="inlineStr">
@@ -4716,7 +4812,7 @@
     <row r="145" ht="14" customHeight="1">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
@@ -4746,7 +4842,7 @@
     <row r="146" ht="14" customHeight="1">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B146" s="5" t="inlineStr">
@@ -4776,7 +4872,7 @@
     <row r="147" ht="14" customHeight="1">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
@@ -4806,7 +4902,7 @@
     <row r="148" ht="14" customHeight="1">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>3B</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B148" s="5" t="inlineStr">
@@ -4924,7 +5020,11 @@
       </c>
     </row>
     <row r="152" ht="14" customHeight="1">
-      <c r="A152" s="11" t="inlineStr"/>
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -4952,7 +5052,7 @@
     <row r="153" ht="14" customHeight="1">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>5C</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -5070,7 +5170,11 @@
       </c>
     </row>
     <row r="157" ht="14" customHeight="1">
-      <c r="A157" s="11" t="inlineStr"/>
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5098,7 +5202,7 @@
     <row r="158" ht="14" customHeight="1">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B158" s="5" t="inlineStr">
@@ -5128,7 +5232,7 @@
     <row r="159" ht="14" customHeight="1">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
@@ -5218,7 +5322,7 @@
     <row r="162" ht="14" customHeight="1">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>5B</t>
         </is>
       </c>
       <c r="B162" s="5" t="inlineStr">
@@ -5246,7 +5350,11 @@
       </c>
     </row>
     <row r="163" ht="14" customHeight="1">
-      <c r="A163" s="11" t="inlineStr"/>
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -5302,7 +5410,11 @@
       </c>
     </row>
     <row r="165" ht="14" customHeight="1">
-      <c r="A165" s="11" t="inlineStr"/>
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>5C</t>
+        </is>
+      </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
@@ -5330,7 +5442,7 @@
     <row r="166" ht="14" customHeight="1">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B166" s="5" t="inlineStr">
@@ -5360,7 +5472,7 @@
     <row r="167" ht="14" customHeight="1">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -5388,7 +5500,11 @@
       </c>
     </row>
     <row r="168" ht="14" customHeight="1">
-      <c r="A168" s="11" t="inlineStr"/>
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
       <c r="B168" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -5414,7 +5530,11 @@
       </c>
     </row>
     <row r="169" ht="14" customHeight="1">
-      <c r="A169" s="11" t="inlineStr"/>
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B169" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -5440,7 +5560,11 @@
       </c>
     </row>
     <row r="170" ht="14" customHeight="1">
-      <c r="A170" s="11" t="inlineStr"/>
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B170" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -5466,7 +5590,11 @@
       </c>
     </row>
     <row r="171" ht="14" customHeight="1">
-      <c r="A171" s="11" t="inlineStr"/>
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -5492,7 +5620,11 @@
       </c>
     </row>
     <row r="172" ht="14" customHeight="1">
-      <c r="A172" s="11" t="inlineStr"/>
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
       <c r="B172" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -5525,11 +5657,7 @@
       </c>
     </row>
     <row r="174" ht="14" customHeight="1">
-      <c r="A174" s="4" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
+      <c r="A174" s="11" t="inlineStr"/>
       <c r="B174" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
@@ -5555,11 +5683,7 @@
       </c>
     </row>
     <row r="175" ht="14" customHeight="1">
-      <c r="A175" s="4" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
+      <c r="A175" s="11" t="inlineStr"/>
       <c r="B175" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
@@ -5585,11 +5709,7 @@
       </c>
     </row>
     <row r="176" ht="14" customHeight="1">
-      <c r="A176" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A176" s="11" t="inlineStr"/>
       <c r="B176" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5615,11 +5735,7 @@
       </c>
     </row>
     <row r="177" ht="14" customHeight="1">
-      <c r="A177" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A177" s="11" t="inlineStr"/>
       <c r="B177" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5671,11 +5787,7 @@
       </c>
     </row>
     <row r="179" ht="14" customHeight="1">
-      <c r="A179" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A179" s="11" t="inlineStr"/>
       <c r="B179" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5701,11 +5813,7 @@
       </c>
     </row>
     <row r="180" ht="14" customHeight="1">
-      <c r="A180" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A180" s="11" t="inlineStr"/>
       <c r="B180" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5757,11 +5865,7 @@
       </c>
     </row>
     <row r="182" ht="14" customHeight="1">
-      <c r="A182" s="4" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
+      <c r="A182" s="11" t="inlineStr"/>
       <c r="B182" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG W</t>
@@ -5787,11 +5891,7 @@
       </c>
     </row>
     <row r="183" ht="14" customHeight="1">
-      <c r="A183" s="4" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
+      <c r="A183" s="11" t="inlineStr"/>
       <c r="B183" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG W</t>
@@ -5817,11 +5917,7 @@
       </c>
     </row>
     <row r="184" ht="14" customHeight="1">
-      <c r="A184" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A184" s="11" t="inlineStr"/>
       <c r="B184" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5847,11 +5943,7 @@
       </c>
     </row>
     <row r="185" ht="14" customHeight="1">
-      <c r="A185" s="4" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
+      <c r="A185" s="11" t="inlineStr"/>
       <c r="B185" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
@@ -5877,11 +5969,7 @@
       </c>
     </row>
     <row r="186" ht="14" customHeight="1">
-      <c r="A186" s="4" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
+      <c r="A186" s="11" t="inlineStr"/>
       <c r="B186" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
@@ -5907,11 +5995,7 @@
       </c>
     </row>
     <row r="187" ht="14" customHeight="1">
-      <c r="A187" s="4" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
+      <c r="A187" s="11" t="inlineStr"/>
       <c r="B187" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
@@ -6024,7 +6108,7 @@
     <row r="192" ht="14" customHeight="1">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B192" s="5" t="inlineStr">
@@ -6084,7 +6168,7 @@
     <row r="194" ht="14" customHeight="1">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>9A</t>
+          <t>6A</t>
         </is>
       </c>
       <c r="B194" s="5" t="inlineStr">
@@ -6144,7 +6228,7 @@
     <row r="196" ht="14" customHeight="1">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>8A</t>
+          <t>6C</t>
         </is>
       </c>
       <c r="B196" s="5" t="inlineStr">
@@ -6202,7 +6286,11 @@
       </c>
     </row>
     <row r="198" ht="14" customHeight="1">
-      <c r="A198" s="11" t="inlineStr"/>
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
           <t>SAMBA GOLF</t>
@@ -6228,7 +6316,11 @@
       </c>
     </row>
     <row r="199" ht="14" customHeight="1">
-      <c r="A199" s="11" t="inlineStr"/>
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B199" s="5" t="inlineStr">
         <is>
           <t>SAMBA GOLF</t>
@@ -6376,7 +6468,7 @@
     <row r="204" ht="14" customHeight="1">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B204" s="5" t="inlineStr">
@@ -6406,7 +6498,7 @@
     <row r="205" ht="14" customHeight="1">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B205" s="5" t="inlineStr">
@@ -6436,7 +6528,7 @@
     <row r="206" ht="14" customHeight="1">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>7A</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B206" s="5" t="inlineStr">
@@ -6494,7 +6586,11 @@
       </c>
     </row>
     <row r="208" ht="14" customHeight="1">
-      <c r="A208" s="11" t="inlineStr"/>
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
       <c r="B208" s="5" t="inlineStr">
         <is>
           <t>GHOST MOTO LOW W</t>
@@ -6552,7 +6648,7 @@
     <row r="210" ht="14" customHeight="1">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>7A</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B210" s="5" t="inlineStr">
@@ -6730,7 +6826,11 @@
       </c>
     </row>
     <row r="216" ht="14" customHeight="1">
-      <c r="A216" s="11" t="inlineStr"/>
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B216" s="5" t="inlineStr">
         <is>
           <t>SAMBA GOLF</t>
@@ -6756,7 +6856,11 @@
       </c>
     </row>
     <row r="217" ht="14" customHeight="1">
-      <c r="A217" s="11" t="inlineStr"/>
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B217" s="5" t="inlineStr">
         <is>
           <t>SAMBA GOLF</t>
@@ -6784,7 +6888,7 @@
     <row r="218" ht="14" customHeight="1">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>6A</t>
         </is>
       </c>
       <c r="B218" s="5" t="inlineStr">
@@ -6812,7 +6916,11 @@
       </c>
     </row>
     <row r="219" ht="14" customHeight="1">
-      <c r="A219" s="11" t="inlineStr"/>
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B219" s="5" t="inlineStr">
         <is>
           <t>SAMBA GOLF</t>
@@ -6840,7 +6948,7 @@
     <row r="220" ht="14" customHeight="1">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>6A</t>
         </is>
       </c>
       <c r="B220" s="5" t="inlineStr">
@@ -6868,7 +6976,11 @@
       </c>
     </row>
     <row r="221" ht="14" customHeight="1">
-      <c r="A221" s="11" t="inlineStr"/>
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B221" s="5" t="inlineStr">
         <is>
           <t>F50 TUNIT MEGA JAH JAH</t>
@@ -6926,7 +7038,7 @@
     <row r="223" ht="14" customHeight="1">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>7A</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B223" s="5" t="inlineStr">
@@ -6956,7 +7068,7 @@
     <row r="224" ht="14" customHeight="1">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>7A</t>
+          <t>6B</t>
         </is>
       </c>
       <c r="B224" s="5" t="inlineStr">
@@ -6984,7 +7096,11 @@
       </c>
     </row>
     <row r="225" ht="14" customHeight="1">
-      <c r="A225" s="11" t="inlineStr"/>
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B225" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -7010,7 +7126,11 @@
       </c>
     </row>
     <row r="226" ht="14" customHeight="1">
-      <c r="A226" s="11" t="inlineStr"/>
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B226" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -7036,7 +7156,11 @@
       </c>
     </row>
     <row r="227" ht="14" customHeight="1">
-      <c r="A227" s="11" t="inlineStr"/>
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B227" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -7062,7 +7186,11 @@
       </c>
     </row>
     <row r="228" ht="14" customHeight="1">
-      <c r="A228" s="11" t="inlineStr"/>
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B228" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -7088,7 +7216,11 @@
       </c>
     </row>
     <row r="229" ht="14" customHeight="1">
-      <c r="A229" s="11" t="inlineStr"/>
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
       <c r="B229" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -7114,7 +7246,11 @@
       </c>
     </row>
     <row r="230" ht="14" customHeight="1">
-      <c r="A230" s="11" t="inlineStr"/>
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
       <c r="B230" s="5" t="inlineStr">
         <is>
           <t>MF2608</t>
@@ -7239,7 +7375,7 @@
     <row r="235" ht="14" customHeight="1">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>7A</t>
         </is>
       </c>
       <c r="B235" s="5" t="inlineStr">
@@ -7299,7 +7435,7 @@
     <row r="237" ht="14" customHeight="1">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>8C</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B237" s="5" t="inlineStr">
@@ -7389,7 +7525,7 @@
     <row r="240" ht="14" customHeight="1">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B240" s="5" t="inlineStr">
@@ -7479,7 +7615,7 @@
     <row r="243" ht="14" customHeight="1">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>7A</t>
         </is>
       </c>
       <c r="B243" s="5" t="inlineStr">
@@ -7689,7 +7825,7 @@
     <row r="250" ht="14" customHeight="1">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>8C</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B250" s="5" t="inlineStr">
@@ -7719,7 +7855,7 @@
     <row r="251" ht="14" customHeight="1">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B251" s="5" t="inlineStr">
@@ -7779,7 +7915,7 @@
     <row r="253" ht="14" customHeight="1">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B253" s="5" t="inlineStr">
@@ -7809,7 +7945,7 @@
     <row r="254" ht="14" customHeight="1">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B254" s="5" t="inlineStr">
@@ -7837,7 +7973,11 @@
       </c>
     </row>
     <row r="255" ht="14" customHeight="1">
-      <c r="A255" s="11" t="inlineStr"/>
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
       <c r="B255" s="5" t="inlineStr">
         <is>
           <t>TOKYO MJ W</t>
@@ -7865,7 +8005,7 @@
     <row r="256" ht="14" customHeight="1">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>8C</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B256" s="5" t="inlineStr">
@@ -7895,7 +8035,7 @@
     <row r="257" ht="14" customHeight="1">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B257" s="5" t="inlineStr">
@@ -7925,7 +8065,7 @@
     <row r="258" ht="14" customHeight="1">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B258" s="5" t="inlineStr">
@@ -7953,7 +8093,11 @@
       </c>
     </row>
     <row r="259" ht="14" customHeight="1">
-      <c r="A259" s="11" t="inlineStr"/>
+      <c r="A259" s="4" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
       <c r="B259" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
@@ -8039,7 +8183,11 @@
       </c>
     </row>
     <row r="262" ht="14" customHeight="1">
-      <c r="A262" s="11" t="inlineStr"/>
+      <c r="A262" s="4" t="inlineStr">
+        <is>
+          <t>7A</t>
+        </is>
+      </c>
       <c r="B262" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -8065,7 +8213,11 @@
       </c>
     </row>
     <row r="263" ht="14" customHeight="1">
-      <c r="A263" s="11" t="inlineStr"/>
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>7A</t>
+        </is>
+      </c>
       <c r="B263" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -8091,7 +8243,11 @@
       </c>
     </row>
     <row r="264" ht="14" customHeight="1">
-      <c r="A264" s="11" t="inlineStr"/>
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>7A</t>
+        </is>
+      </c>
       <c r="B264" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -8246,7 +8402,7 @@
     <row r="270" ht="14" customHeight="1">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B270" s="5" t="inlineStr">
@@ -8336,7 +8492,7 @@
     <row r="273" ht="14" customHeight="1">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B273" s="5" t="inlineStr">
@@ -8426,7 +8582,7 @@
     <row r="276" ht="14" customHeight="1">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>10B</t>
+          <t>8A</t>
         </is>
       </c>
       <c r="B276" s="5" t="inlineStr">
@@ -8516,7 +8672,7 @@
     <row r="279" ht="14" customHeight="1">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B279" s="5" t="inlineStr">
@@ -8816,7 +8972,7 @@
     <row r="289" ht="14" customHeight="1">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B289" s="5" t="inlineStr">
@@ -8876,7 +9032,7 @@
     <row r="291" ht="14" customHeight="1">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B291" s="5" t="inlineStr">
@@ -8906,7 +9062,7 @@
     <row r="292" ht="14" customHeight="1">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>8A</t>
         </is>
       </c>
       <c r="B292" s="5" t="inlineStr">
@@ -8934,7 +9090,11 @@
       </c>
     </row>
     <row r="293" ht="14" customHeight="1">
-      <c r="A293" s="11" t="inlineStr"/>
+      <c r="A293" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B293" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -8962,7 +9122,7 @@
     <row r="294" ht="14" customHeight="1">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>8A</t>
         </is>
       </c>
       <c r="B294" s="5" t="inlineStr">
@@ -8990,7 +9150,11 @@
       </c>
     </row>
     <row r="295" ht="14" customHeight="1">
-      <c r="A295" s="11" t="inlineStr"/>
+      <c r="A295" s="4" t="inlineStr">
+        <is>
+          <t>8C</t>
+        </is>
+      </c>
       <c r="B295" s="5" t="inlineStr">
         <is>
           <t>TOKYO MJ W</t>
@@ -9168,7 +9332,7 @@
     <row r="301" ht="14" customHeight="1">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>8A</t>
         </is>
       </c>
       <c r="B301" s="5" t="inlineStr">
@@ -9196,7 +9360,11 @@
       </c>
     </row>
     <row r="302" ht="14" customHeight="1">
-      <c r="A302" s="11" t="inlineStr"/>
+      <c r="A302" s="4" t="inlineStr">
+        <is>
+          <t>8C</t>
+        </is>
+      </c>
       <c r="B302" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
@@ -9222,7 +9390,11 @@
       </c>
     </row>
     <row r="303" ht="14" customHeight="1">
-      <c r="A303" s="11" t="inlineStr"/>
+      <c r="A303" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B303" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -9248,7 +9420,11 @@
       </c>
     </row>
     <row r="304" ht="14" customHeight="1">
-      <c r="A304" s="11" t="inlineStr"/>
+      <c r="A304" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B304" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -9274,7 +9450,11 @@
       </c>
     </row>
     <row r="305" ht="14" customHeight="1">
-      <c r="A305" s="11" t="inlineStr"/>
+      <c r="A305" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B305" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -9300,7 +9480,11 @@
       </c>
     </row>
     <row r="306" ht="14" customHeight="1">
-      <c r="A306" s="11" t="inlineStr"/>
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B306" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -9326,7 +9510,11 @@
       </c>
     </row>
     <row r="307" ht="14" customHeight="1">
-      <c r="A307" s="11" t="inlineStr"/>
+      <c r="A307" s="4" t="inlineStr">
+        <is>
+          <t>8A</t>
+        </is>
+      </c>
       <c r="B307" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -9449,7 +9637,11 @@
       </c>
     </row>
     <row r="312" ht="14" customHeight="1">
-      <c r="A312" s="11" t="inlineStr"/>
+      <c r="A312" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B312" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
@@ -9475,7 +9667,11 @@
       </c>
     </row>
     <row r="313" ht="14" customHeight="1">
-      <c r="A313" s="11" t="inlineStr"/>
+      <c r="A313" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B313" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
@@ -9773,7 +9969,7 @@
     <row r="323" ht="14" customHeight="1">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>9B</t>
         </is>
       </c>
       <c r="B323" s="5" t="inlineStr">
@@ -10221,7 +10417,11 @@
       </c>
     </row>
     <row r="338" ht="14" customHeight="1">
-      <c r="A338" s="11" t="inlineStr"/>
+      <c r="A338" s="4" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
       <c r="B338" s="5" t="inlineStr">
         <is>
           <t>SL 72 OG W</t>
@@ -10279,7 +10479,7 @@
     <row r="340" ht="14" customHeight="1">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>9B</t>
         </is>
       </c>
       <c r="B340" s="5" t="inlineStr">
@@ -10309,7 +10509,7 @@
     <row r="341" ht="14" customHeight="1">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>10B</t>
+          <t>9A</t>
         </is>
       </c>
       <c r="B341" s="5" t="inlineStr">
@@ -10427,7 +10627,11 @@
       </c>
     </row>
     <row r="345" ht="14" customHeight="1">
-      <c r="A345" s="11" t="inlineStr"/>
+      <c r="A345" s="4" t="inlineStr">
+        <is>
+          <t>9B</t>
+        </is>
+      </c>
       <c r="B345" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0</t>
@@ -10455,7 +10659,7 @@
     <row r="346" ht="14" customHeight="1">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>9B</t>
         </is>
       </c>
       <c r="B346" s="5" t="inlineStr">
@@ -10483,7 +10687,11 @@
       </c>
     </row>
     <row r="347" ht="14" customHeight="1">
-      <c r="A347" s="11" t="inlineStr"/>
+      <c r="A347" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B347" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -10509,7 +10717,11 @@
       </c>
     </row>
     <row r="348" ht="14" customHeight="1">
-      <c r="A348" s="11" t="inlineStr"/>
+      <c r="A348" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B348" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -10535,7 +10747,11 @@
       </c>
     </row>
     <row r="349" ht="14" customHeight="1">
-      <c r="A349" s="11" t="inlineStr"/>
+      <c r="A349" s="4" t="inlineStr">
+        <is>
+          <t>9B</t>
+        </is>
+      </c>
       <c r="B349" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -10561,7 +10777,11 @@
       </c>
     </row>
     <row r="350" ht="14" customHeight="1">
-      <c r="A350" s="11" t="inlineStr"/>
+      <c r="A350" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B350" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -10587,7 +10807,11 @@
       </c>
     </row>
     <row r="351" ht="14" customHeight="1">
-      <c r="A351" s="11" t="inlineStr"/>
+      <c r="A351" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
       <c r="B351" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -10622,7 +10846,7 @@
     <row r="353" ht="14" customHeight="1">
       <c r="A353" s="4" t="inlineStr">
         <is>
-          <t>9A</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="B353" s="5" t="inlineStr">
@@ -10650,7 +10874,11 @@
       </c>
     </row>
     <row r="354" ht="14" customHeight="1">
-      <c r="A354" s="11" t="inlineStr"/>
+      <c r="A354" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B354" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
@@ -10676,7 +10904,11 @@
       </c>
     </row>
     <row r="355" ht="14" customHeight="1">
-      <c r="A355" s="11" t="inlineStr"/>
+      <c r="A355" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B355" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
@@ -11032,7 +11264,11 @@
       </c>
     </row>
     <row r="367" ht="14" customHeight="1">
-      <c r="A367" s="11" t="inlineStr"/>
+      <c r="A367" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B367" s="5" t="inlineStr">
         <is>
           <t>SPEZIAL GOLF</t>
@@ -11058,7 +11294,11 @@
       </c>
     </row>
     <row r="368" ht="14" customHeight="1">
-      <c r="A368" s="11" t="inlineStr"/>
+      <c r="A368" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B368" s="5" t="inlineStr">
         <is>
           <t>SPEZIAL GOLF</t>
@@ -11084,7 +11324,11 @@
       </c>
     </row>
     <row r="369" ht="14" customHeight="1">
-      <c r="A369" s="11" t="inlineStr"/>
+      <c r="A369" s="4" t="inlineStr">
+        <is>
+          <t>10B</t>
+        </is>
+      </c>
       <c r="B369" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -11110,7 +11354,11 @@
       </c>
     </row>
     <row r="370" ht="14" customHeight="1">
-      <c r="A370" s="11" t="inlineStr"/>
+      <c r="A370" s="4" t="inlineStr">
+        <is>
+          <t>10B</t>
+        </is>
+      </c>
       <c r="B370" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -11226,7 +11474,11 @@
       </c>
     </row>
     <row r="374" ht="14" customHeight="1">
-      <c r="A374" s="11" t="inlineStr"/>
+      <c r="A374" s="4" t="inlineStr">
+        <is>
+          <t>10B</t>
+        </is>
+      </c>
       <c r="B374" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -11282,7 +11534,11 @@
       </c>
     </row>
     <row r="376" ht="14" customHeight="1">
-      <c r="A376" s="11" t="inlineStr"/>
+      <c r="A376" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B376" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
@@ -11308,7 +11564,11 @@
       </c>
     </row>
     <row r="377" ht="14" customHeight="1">
-      <c r="A377" s="11" t="inlineStr"/>
+      <c r="A377" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B377" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
@@ -11484,7 +11744,11 @@
       </c>
     </row>
     <row r="383" ht="14" customHeight="1">
-      <c r="A383" s="11" t="inlineStr"/>
+      <c r="A383" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B383" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
@@ -11512,7 +11776,7 @@
     <row r="384" ht="14" customHeight="1">
       <c r="A384" s="4" t="inlineStr">
         <is>
-          <t>10B</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="B384" s="5" t="inlineStr">
@@ -11542,7 +11806,7 @@
     <row r="385" ht="14" customHeight="1">
       <c r="A385" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>10B</t>
         </is>
       </c>
       <c r="B385" s="5" t="inlineStr">
@@ -11572,7 +11836,7 @@
     <row r="386" ht="14" customHeight="1">
       <c r="A386" s="4" t="inlineStr">
         <is>
-          <t>5B</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="B386" s="5" t="inlineStr">
@@ -11600,7 +11864,11 @@
       </c>
     </row>
     <row r="387" ht="14" customHeight="1">
-      <c r="A387" s="11" t="inlineStr"/>
+      <c r="A387" s="4" t="inlineStr">
+        <is>
+          <t>10B</t>
+        </is>
+      </c>
       <c r="B387" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -11626,7 +11894,11 @@
       </c>
     </row>
     <row r="388" ht="14" customHeight="1">
-      <c r="A388" s="11" t="inlineStr"/>
+      <c r="A388" s="4" t="inlineStr">
+        <is>
+          <t>10C</t>
+        </is>
+      </c>
       <c r="B388" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
@@ -11682,7 +11954,11 @@
       </c>
     </row>
     <row r="390" ht="14" customHeight="1">
-      <c r="A390" s="11" t="inlineStr"/>
+      <c r="A390" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B390" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -11708,7 +11984,11 @@
       </c>
     </row>
     <row r="391" ht="14" customHeight="1">
-      <c r="A391" s="11" t="inlineStr"/>
+      <c r="A391" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B391" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -11734,7 +12014,11 @@
       </c>
     </row>
     <row r="392" ht="14" customHeight="1">
-      <c r="A392" s="11" t="inlineStr"/>
+      <c r="A392" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B392" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -11760,7 +12044,11 @@
       </c>
     </row>
     <row r="393" ht="14" customHeight="1">
-      <c r="A393" s="11" t="inlineStr"/>
+      <c r="A393" s="4" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
       <c r="B393" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -11855,7 +12143,7 @@
     <row r="397" ht="14" customHeight="1">
       <c r="A397" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B397" s="5" t="inlineStr">
@@ -12035,7 +12323,7 @@
     <row r="403" ht="14" customHeight="1">
       <c r="A403" s="4" t="inlineStr">
         <is>
-          <t>11B1</t>
+          <t>11A1</t>
         </is>
       </c>
       <c r="B403" s="5" t="inlineStr">
@@ -12093,7 +12381,11 @@
       </c>
     </row>
     <row r="405" ht="14" customHeight="1">
-      <c r="A405" s="11" t="inlineStr"/>
+      <c r="A405" s="4" t="inlineStr">
+        <is>
+          <t>11A1</t>
+        </is>
+      </c>
       <c r="B405" s="5" t="inlineStr">
         <is>
           <t>ADIPOWER 26 SL BOA</t>
@@ -12119,7 +12411,11 @@
       </c>
     </row>
     <row r="406" ht="14" customHeight="1">
-      <c r="A406" s="11" t="inlineStr"/>
+      <c r="A406" s="4" t="inlineStr">
+        <is>
+          <t>11A1</t>
+        </is>
+      </c>
       <c r="B406" s="5" t="inlineStr">
         <is>
           <t>ADIPOWER 26 SL BOA</t>
@@ -12777,7 +13073,7 @@
     <row r="428" ht="14" customHeight="1">
       <c r="A428" s="4" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>11A2</t>
         </is>
       </c>
       <c r="B428" s="5" t="inlineStr">
@@ -12865,7 +13161,11 @@
       </c>
     </row>
     <row r="431" ht="14" customHeight="1">
-      <c r="A431" s="11" t="inlineStr"/>
+      <c r="A431" s="4" t="inlineStr">
+        <is>
+          <t>11A1</t>
+        </is>
+      </c>
       <c r="B431" s="5" t="inlineStr">
         <is>
           <t>ADIPOWER 26 SL BOA</t>
@@ -12951,7 +13251,11 @@
       </c>
     </row>
     <row r="434" ht="14" customHeight="1">
-      <c r="A434" s="11" t="inlineStr"/>
+      <c r="A434" s="4" t="inlineStr">
+        <is>
+          <t>11B1</t>
+        </is>
+      </c>
       <c r="B434" s="5" t="inlineStr">
         <is>
           <t>W S2G 26 LEATHER</t>
@@ -12977,7 +13281,11 @@
       </c>
     </row>
     <row r="435" ht="14" customHeight="1">
-      <c r="A435" s="11" t="inlineStr"/>
+      <c r="A435" s="4" t="inlineStr">
+        <is>
+          <t>11B1</t>
+        </is>
+      </c>
       <c r="B435" s="5" t="inlineStr">
         <is>
           <t>W S2G 26 LEATHER</t>
@@ -13095,7 +13403,7 @@
     <row r="439" ht="14" customHeight="1">
       <c r="A439" s="4" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>11B1</t>
         </is>
       </c>
       <c r="B439" s="5" t="inlineStr">
@@ -13123,7 +13431,11 @@
       </c>
     </row>
     <row r="440" ht="14" customHeight="1">
-      <c r="A440" s="11" t="inlineStr"/>
+      <c r="A440" s="4" t="inlineStr">
+        <is>
+          <t>11A1</t>
+        </is>
+      </c>
       <c r="B440" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -13149,7 +13461,11 @@
       </c>
     </row>
     <row r="441" ht="14" customHeight="1">
-      <c r="A441" s="11" t="inlineStr"/>
+      <c r="A441" s="4" t="inlineStr">
+        <is>
+          <t>11A1</t>
+        </is>
+      </c>
       <c r="B441" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -13424,7 +13740,7 @@
     <row r="451" ht="14" customHeight="1">
       <c r="A451" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>11C</t>
         </is>
       </c>
       <c r="B451" s="5" t="inlineStr">
@@ -13454,7 +13770,7 @@
     <row r="452" ht="14" customHeight="1">
       <c r="A452" s="4" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>11B2</t>
         </is>
       </c>
       <c r="B452" s="5" t="inlineStr">
@@ -13482,7 +13798,11 @@
       </c>
     </row>
     <row r="453" ht="14" customHeight="1">
-      <c r="A453" s="11" t="inlineStr"/>
+      <c r="A453" s="4" t="inlineStr">
+        <is>
+          <t>11C</t>
+        </is>
+      </c>
       <c r="B453" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -13538,7 +13858,11 @@
       </c>
     </row>
     <row r="455" ht="14" customHeight="1">
-      <c r="A455" s="11" t="inlineStr"/>
+      <c r="A455" s="4" t="inlineStr">
+        <is>
+          <t>11B2</t>
+        </is>
+      </c>
       <c r="B455" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -13564,7 +13888,11 @@
       </c>
     </row>
     <row r="456" ht="14" customHeight="1">
-      <c r="A456" s="11" t="inlineStr"/>
+      <c r="A456" s="4" t="inlineStr">
+        <is>
+          <t>11C</t>
+        </is>
+      </c>
       <c r="B456" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -13590,7 +13918,11 @@
       </c>
     </row>
     <row r="457" ht="14" customHeight="1">
-      <c r="A457" s="11" t="inlineStr"/>
+      <c r="A457" s="4" t="inlineStr">
+        <is>
+          <t>11C</t>
+        </is>
+      </c>
       <c r="B457" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -13616,7 +13948,11 @@
       </c>
     </row>
     <row r="458" ht="14" customHeight="1">
-      <c r="A458" s="11" t="inlineStr"/>
+      <c r="A458" s="4" t="inlineStr">
+        <is>
+          <t>11B2</t>
+        </is>
+      </c>
       <c r="B458" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -13642,7 +13978,11 @@
       </c>
     </row>
     <row r="459" ht="14" customHeight="1">
-      <c r="A459" s="11" t="inlineStr"/>
+      <c r="A459" s="4" t="inlineStr">
+        <is>
+          <t>11B2</t>
+        </is>
+      </c>
       <c r="B459" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -13767,7 +14107,7 @@
     <row r="464" ht="14" customHeight="1">
       <c r="A464" s="4" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="B464" s="5" t="inlineStr">
@@ -13797,7 +14137,7 @@
     <row r="465" ht="14" customHeight="1">
       <c r="A465" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>12A</t>
         </is>
       </c>
       <c r="B465" s="5" t="inlineStr">
@@ -13915,7 +14255,11 @@
       </c>
     </row>
     <row r="469" ht="14" customHeight="1">
-      <c r="A469" s="11" t="inlineStr"/>
+      <c r="A469" s="4" t="inlineStr">
+        <is>
+          <t>12A</t>
+        </is>
+      </c>
       <c r="B469" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
@@ -13971,7 +14315,11 @@
       </c>
     </row>
     <row r="471" ht="14" customHeight="1">
-      <c r="A471" s="11" t="inlineStr"/>
+      <c r="A471" s="4" t="inlineStr">
+        <is>
+          <t>12A</t>
+        </is>
+      </c>
       <c r="B471" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
@@ -14027,7 +14375,11 @@
       </c>
     </row>
     <row r="473" ht="14" customHeight="1">
-      <c r="A473" s="11" t="inlineStr"/>
+      <c r="A473" s="4" t="inlineStr">
+        <is>
+          <t>12A</t>
+        </is>
+      </c>
       <c r="B473" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
@@ -14055,7 +14407,7 @@
     <row r="474" ht="14" customHeight="1">
       <c r="A474" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>12A</t>
         </is>
       </c>
       <c r="B474" s="5" t="inlineStr">
@@ -14083,7 +14435,11 @@
       </c>
     </row>
     <row r="475" ht="14" customHeight="1">
-      <c r="A475" s="11" t="inlineStr"/>
+      <c r="A475" s="4" t="inlineStr">
+        <is>
+          <t>12C</t>
+        </is>
+      </c>
       <c r="B475" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -14141,7 +14497,7 @@
     <row r="477" ht="14" customHeight="1">
       <c r="A477" s="4" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="B477" s="5" t="inlineStr">
@@ -14171,7 +14527,7 @@
     <row r="478" ht="14" customHeight="1">
       <c r="A478" s="4" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>12D</t>
         </is>
       </c>
       <c r="B478" s="5" t="inlineStr">
@@ -14229,7 +14585,11 @@
       </c>
     </row>
     <row r="480" ht="14" customHeight="1">
-      <c r="A480" s="11" t="inlineStr"/>
+      <c r="A480" s="4" t="inlineStr">
+        <is>
+          <t>12D</t>
+        </is>
+      </c>
       <c r="B480" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -14255,7 +14615,11 @@
       </c>
     </row>
     <row r="481" ht="14" customHeight="1">
-      <c r="A481" s="11" t="inlineStr"/>
+      <c r="A481" s="4" t="inlineStr">
+        <is>
+          <t>12D</t>
+        </is>
+      </c>
       <c r="B481" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -14281,7 +14645,11 @@
       </c>
     </row>
     <row r="482" ht="14" customHeight="1">
-      <c r="A482" s="11" t="inlineStr"/>
+      <c r="A482" s="4" t="inlineStr">
+        <is>
+          <t>12D</t>
+        </is>
+      </c>
       <c r="B482" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 W</t>
@@ -14309,7 +14677,7 @@
     <row r="483" ht="14" customHeight="1">
       <c r="A483" s="4" t="inlineStr">
         <is>
-          <t>5B</t>
+          <t>12D</t>
         </is>
       </c>
       <c r="B483" s="5" t="inlineStr">
@@ -14339,7 +14707,7 @@
     <row r="484" ht="14" customHeight="1">
       <c r="A484" s="4" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="B484" s="5" t="inlineStr">
@@ -14367,7 +14735,11 @@
       </c>
     </row>
     <row r="485" ht="14" customHeight="1">
-      <c r="A485" s="11" t="inlineStr"/>
+      <c r="A485" s="4" t="inlineStr">
+        <is>
+          <t>12C</t>
+        </is>
+      </c>
       <c r="B485" s="5" t="inlineStr">
         <is>
           <t>MF2603</t>
@@ -14393,7 +14765,11 @@
       </c>
     </row>
     <row r="486" ht="14" customHeight="1">
-      <c r="A486" s="11" t="inlineStr"/>
+      <c r="A486" s="4" t="inlineStr">
+        <is>
+          <t>12C</t>
+        </is>
+      </c>
       <c r="B486" s="5" t="inlineStr">
         <is>
           <t>MF2604</t>
@@ -14419,7 +14795,11 @@
       </c>
     </row>
     <row r="487" ht="14" customHeight="1">
-      <c r="A487" s="11" t="inlineStr"/>
+      <c r="A487" s="4" t="inlineStr">
+        <is>
+          <t>12C</t>
+        </is>
+      </c>
       <c r="B487" s="5" t="inlineStr">
         <is>
           <t>MF2605</t>
@@ -14445,7 +14825,11 @@
       </c>
     </row>
     <row r="488" ht="14" customHeight="1">
-      <c r="A488" s="11" t="inlineStr"/>
+      <c r="A488" s="4" t="inlineStr">
+        <is>
+          <t>12A</t>
+        </is>
+      </c>
       <c r="B488" s="5" t="inlineStr">
         <is>
           <t>MF2606</t>
@@ -14471,7 +14855,11 @@
       </c>
     </row>
     <row r="489" ht="14" customHeight="1">
-      <c r="A489" s="11" t="inlineStr"/>
+      <c r="A489" s="4" t="inlineStr">
+        <is>
+          <t>12A</t>
+        </is>
+      </c>
       <c r="B489" s="5" t="inlineStr">
         <is>
           <t>MF2607</t>
@@ -14504,11 +14892,7 @@
       </c>
     </row>
     <row r="491" ht="14" customHeight="1">
-      <c r="A491" s="4" t="inlineStr">
-        <is>
-          <t>6C</t>
-        </is>
-      </c>
+      <c r="A491" s="11" t="inlineStr"/>
       <c r="B491" s="5" t="inlineStr">
         <is>
           <t>SAMBA</t>
@@ -14534,11 +14918,7 @@
       </c>
     </row>
     <row r="492" ht="14" customHeight="1">
-      <c r="A492" s="4" t="inlineStr">
-        <is>
-          <t>8A</t>
-        </is>
-      </c>
+      <c r="A492" s="11" t="inlineStr"/>
       <c r="B492" s="5" t="inlineStr">
         <is>
           <t>SAMBA</t>
@@ -14616,11 +14996,7 @@
       </c>
     </row>
     <row r="495" ht="14" customHeight="1">
-      <c r="A495" s="4" t="inlineStr">
-        <is>
-          <t>10B</t>
-        </is>
-      </c>
+      <c r="A495" s="11" t="inlineStr"/>
       <c r="B495" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -14646,11 +15022,7 @@
       </c>
     </row>
     <row r="496" ht="14" customHeight="1">
-      <c r="A496" s="4" t="inlineStr">
-        <is>
-          <t>9B</t>
-        </is>
-      </c>
+      <c r="A496" s="11" t="inlineStr"/>
       <c r="B496" s="5" t="inlineStr">
         <is>
           <t>ADISTAR XLG 2.0 J</t>
@@ -14813,11 +15185,7 @@
       </c>
     </row>
     <row r="503" ht="14" customHeight="1">
-      <c r="A503" s="4" t="inlineStr">
-        <is>
-          <t>2C</t>
-        </is>
-      </c>
+      <c r="A503" s="11" t="inlineStr"/>
       <c r="B503" s="5" t="inlineStr">
         <is>
           <t>RETROCROSS 25</t>
@@ -14843,11 +15211,7 @@
       </c>
     </row>
     <row r="504" ht="14" customHeight="1">
-      <c r="A504" s="4" t="inlineStr">
-        <is>
-          <t>8A</t>
-        </is>
-      </c>
+      <c r="A504" s="11" t="inlineStr"/>
       <c r="B504" s="5" t="inlineStr">
         <is>
           <t>SAMBA</t>
@@ -14873,11 +15237,7 @@
       </c>
     </row>
     <row r="505" ht="14" customHeight="1">
-      <c r="A505" s="4" t="inlineStr">
-        <is>
-          <t>2C</t>
-        </is>
-      </c>
+      <c r="A505" s="11" t="inlineStr"/>
       <c r="B505" s="5" t="inlineStr">
         <is>
           <t>RETROCROSS 25</t>
@@ -14903,11 +15263,7 @@
       </c>
     </row>
     <row r="506" ht="14" customHeight="1">
-      <c r="A506" s="4" t="inlineStr">
-        <is>
-          <t>2C</t>
-        </is>
-      </c>
+      <c r="A506" s="11" t="inlineStr"/>
       <c r="B506" s="5" t="inlineStr">
         <is>
           <t>RETROCROSS 25</t>
@@ -14933,11 +15289,7 @@
       </c>
     </row>
     <row r="507" ht="14" customHeight="1">
-      <c r="A507" s="4" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
+      <c r="A507" s="11" t="inlineStr"/>
       <c r="B507" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
@@ -14963,11 +15315,7 @@
       </c>
     </row>
     <row r="508" ht="14" customHeight="1">
-      <c r="A508" s="4" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
+      <c r="A508" s="11" t="inlineStr"/>
       <c r="B508" s="5" t="inlineStr">
         <is>
           <t>MEGARIDE F50</t>

</xml_diff>